<commit_message>
feat(setup): add final setup excel templates for dormitories, classes, and santri
</commit_message>
<xml_diff>
--- a/Setup_1_Asrama_Putra_v2.xlsx
+++ b/Setup_1_Asrama_Putra_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ambisss\My Projek Laravel\elf_v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B89CD67C-7B94-426E-A49B-1374F9C5EF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C9D2343-9B82-4DE1-864C-3BD9EF27C96A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
   <si>
     <t>Nama Komplek *</t>
   </si>
@@ -98,6 +98,12 @@
   </si>
   <si>
     <t>Kamar 17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dalem Etan </t>
+  </si>
+  <si>
+    <t>Kamar 18</t>
   </si>
 </sst>
 </file>
@@ -135,7 +141,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -173,16 +179,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -489,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -750,6 +770,20 @@
         <v>15</v>
       </c>
     </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="2">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>